<commit_message>
Rank the charts that claim a ranking
The Pareto was not the only one. Three more charts sorted nothing and plotted
rows in whatever order somebody typed them:

  * The X-Y matrix, titled "the tall bars are where to look", made you scan for
    the tall bar.
  * The solution selection matrix ranked nothing.
  * The FMEA, whose entire method is "work the highest RPN first", buried the
    worst failure mode wherever it happened to be entered. It now reads
    504, 432, 336, 288, 168, 105 — highest risk first, which is the only order
    an FMEA is meant to be read in.

Built once as ranked_block() in chart_specs.py and applied to all three: a
tie-broken RANK beside the source table, then INDEX/MATCH resolving each
position into a block the chart plots. No macros, no re-typing, and it re-ranks
itself the moment a score changes.

verify.py now recalculates all three and fails unless the plotted values come
out in descending order.
</commit_message>
<xml_diff>
--- a/templates/11-cause-effect-xy-matrix.xlsx
+++ b/templates/11-cause-effect-xy-matrix.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -160,6 +160,11 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF6B7280"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -255,7 +260,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -397,6 +402,10 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -483,7 +492,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Weighted total by candidate cause — the tall bars are where to look</a:t>
+              <a:t>Weighted total by candidate cause — ranked, tallest first</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -507,12 +516,12 @@
           <invertIfNegative val="0"/>
           <cat>
             <numRef>
-              <f>'X-Y matrix'!$A$15:$A$36</f>
+              <f>'X-Y matrix'!$M$15:$M$36</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'X-Y matrix'!$H$15:$H$36</f>
+              <f>'X-Y matrix'!$N$15:$N$36</f>
             </numRef>
           </val>
         </ser>
@@ -546,7 +555,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'X-Y matrix'!$J$15:$J$36</f>
+              <f>'X-Y matrix'!$O$15:$O$36</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -596,7 +605,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>13</row>
       <rowOff>0</rowOff>
@@ -932,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="22" min="1" max="1"/>
@@ -1118,6 +1127,31 @@
           <t>Mean</t>
         </is>
       </c>
+      <c r="K14" s="49" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="L14" s="47" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="M14" s="47" t="inlineStr">
+        <is>
+          <t>Candidate cause</t>
+        </is>
+      </c>
+      <c r="N14" s="47" t="inlineStr">
+        <is>
+          <t>Weighted total</t>
+        </is>
+      </c>
+      <c r="O14" s="47" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="23">
       <c r="A15" s="45" t="inlineStr">
@@ -1157,6 +1191,25 @@
         <f>IF(H15="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K15" s="50">
+        <f>IF(H15="","",RANK(H15,$H$15:$H$36,0)+COUNTIF($H$15:H15,H15)-1)</f>
+        <v/>
+      </c>
+      <c r="L15" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L15,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L15,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="48">
+        <f>IF(N15="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1" s="23">
       <c r="A16" s="46" t="inlineStr">
@@ -1196,6 +1249,25 @@
         <f>IF(H16="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K16" s="50">
+        <f>IF(H16="","",RANK(H16,$H$15:$H$36,0)+COUNTIF($H$15:H16,H16)-1)</f>
+        <v/>
+      </c>
+      <c r="L16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L16,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L16,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="48">
+        <f>IF(N16="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="23">
       <c r="A17" s="46" t="inlineStr">
@@ -1235,6 +1307,25 @@
         <f>IF(H17="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K17" s="50">
+        <f>IF(H17="","",RANK(H17,$H$15:$H$36,0)+COUNTIF($H$15:H17,H17)-1)</f>
+        <v/>
+      </c>
+      <c r="L17" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="M17" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L17,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L17,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="48">
+        <f>IF(N17="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1" s="23">
       <c r="A18" s="46" t="inlineStr">
@@ -1274,6 +1365,25 @@
         <f>IF(H18="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K18" s="50">
+        <f>IF(H18="","",RANK(H18,$H$15:$H$36,0)+COUNTIF($H$15:H18,H18)-1)</f>
+        <v/>
+      </c>
+      <c r="L18" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="M18" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L18,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L18,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="48">
+        <f>IF(N18="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1" s="23">
       <c r="A19" s="46" t="inlineStr">
@@ -1313,6 +1423,25 @@
         <f>IF(H19="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K19" s="50">
+        <f>IF(H19="","",RANK(H19,$H$15:$H$36,0)+COUNTIF($H$15:H19,H19)-1)</f>
+        <v/>
+      </c>
+      <c r="L19" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L19,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L19,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="48">
+        <f>IF(N19="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1" s="23">
       <c r="A20" s="46" t="inlineStr">
@@ -1352,6 +1481,25 @@
         <f>IF(H20="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K20" s="50">
+        <f>IF(H20="","",RANK(H20,$H$15:$H$36,0)+COUNTIF($H$15:H20,H20)-1)</f>
+        <v/>
+      </c>
+      <c r="L20" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="M20" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L20,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L20,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="48">
+        <f>IF(N20="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1" s="23">
       <c r="A21" s="46" t="inlineStr">
@@ -1391,6 +1539,25 @@
         <f>IF(H21="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K21" s="50">
+        <f>IF(H21="","",RANK(H21,$H$15:$H$36,0)+COUNTIF($H$15:H21,H21)-1)</f>
+        <v/>
+      </c>
+      <c r="L21" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="M21" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L21,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L21,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="48">
+        <f>IF(N21="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1" s="23">
       <c r="A22" s="46" t="inlineStr">
@@ -1428,6 +1595,25 @@
       </c>
       <c r="J22" s="48">
         <f>IF(H22="","",AVERAGE($H$15:$H$36))</f>
+        <v/>
+      </c>
+      <c r="K22" s="50">
+        <f>IF(H22="","",RANK(H22,$H$15:$H$36,0)+COUNTIF($H$15:H22,H22)-1)</f>
+        <v/>
+      </c>
+      <c r="L22" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="M22" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L22,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L22,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="48">
+        <f>IF(N22="","",AVERAGE($N$15:$N$36))</f>
         <v/>
       </c>
     </row>
@@ -1451,6 +1637,25 @@
         <f>IF(H23="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K23" s="50">
+        <f>IF(H23="","",RANK(H23,$H$15:$H$36,0)+COUNTIF($H$15:H23,H23)-1)</f>
+        <v/>
+      </c>
+      <c r="L23" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="M23" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L23,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L23,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="48">
+        <f>IF(N23="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="23">
       <c r="A24" s="43" t="n"/>
@@ -1472,6 +1677,25 @@
         <f>IF(H24="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K24" s="50">
+        <f>IF(H24="","",RANK(H24,$H$15:$H$36,0)+COUNTIF($H$15:H24,H24)-1)</f>
+        <v/>
+      </c>
+      <c r="L24" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="M24" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L24,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L24,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="48">
+        <f>IF(N24="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="23">
       <c r="A25" s="43" t="n"/>
@@ -1493,6 +1717,25 @@
         <f>IF(H25="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K25" s="50">
+        <f>IF(H25="","",RANK(H25,$H$15:$H$36,0)+COUNTIF($H$15:H25,H25)-1)</f>
+        <v/>
+      </c>
+      <c r="L25" s="51" t="n">
+        <v>11</v>
+      </c>
+      <c r="M25" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L25,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L25,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="48">
+        <f>IF(N25="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1" s="23">
       <c r="A26" s="43" t="n"/>
@@ -1514,6 +1757,25 @@
         <f>IF(H26="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K26" s="50">
+        <f>IF(H26="","",RANK(H26,$H$15:$H$36,0)+COUNTIF($H$15:H26,H26)-1)</f>
+        <v/>
+      </c>
+      <c r="L26" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="M26" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L26,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L26,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="48">
+        <f>IF(N26="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1" s="23">
       <c r="A27" s="43" t="n"/>
@@ -1535,6 +1797,25 @@
         <f>IF(H27="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K27" s="50">
+        <f>IF(H27="","",RANK(H27,$H$15:$H$36,0)+COUNTIF($H$15:H27,H27)-1)</f>
+        <v/>
+      </c>
+      <c r="L27" s="51" t="n">
+        <v>13</v>
+      </c>
+      <c r="M27" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L27,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L27,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="48">
+        <f>IF(N27="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1" s="23">
       <c r="A28" s="43" t="n"/>
@@ -1556,6 +1837,25 @@
         <f>IF(H28="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K28" s="50">
+        <f>IF(H28="","",RANK(H28,$H$15:$H$36,0)+COUNTIF($H$15:H28,H28)-1)</f>
+        <v/>
+      </c>
+      <c r="L28" s="51" t="n">
+        <v>14</v>
+      </c>
+      <c r="M28" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L28,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L28,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O28" s="48">
+        <f>IF(N28="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1" s="23">
       <c r="A29" s="43" t="n"/>
@@ -1577,6 +1877,25 @@
         <f>IF(H29="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K29" s="50">
+        <f>IF(H29="","",RANK(H29,$H$15:$H$36,0)+COUNTIF($H$15:H29,H29)-1)</f>
+        <v/>
+      </c>
+      <c r="L29" s="51" t="n">
+        <v>15</v>
+      </c>
+      <c r="M29" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L29,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N29" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L29,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O29" s="48">
+        <f>IF(N29="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1" s="23">
       <c r="A30" s="43" t="n"/>
@@ -1598,6 +1917,25 @@
         <f>IF(H30="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K30" s="50">
+        <f>IF(H30="","",RANK(H30,$H$15:$H$36,0)+COUNTIF($H$15:H30,H30)-1)</f>
+        <v/>
+      </c>
+      <c r="L30" s="51" t="n">
+        <v>16</v>
+      </c>
+      <c r="M30" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L30,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N30" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L30,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O30" s="48">
+        <f>IF(N30="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1" s="23">
       <c r="A31" s="43" t="n"/>
@@ -1619,6 +1957,25 @@
         <f>IF(H31="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K31" s="50">
+        <f>IF(H31="","",RANK(H31,$H$15:$H$36,0)+COUNTIF($H$15:H31,H31)-1)</f>
+        <v/>
+      </c>
+      <c r="L31" s="51" t="n">
+        <v>17</v>
+      </c>
+      <c r="M31" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L31,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N31" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L31,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O31" s="48">
+        <f>IF(N31="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="23">
       <c r="A32" s="43" t="n"/>
@@ -1640,6 +1997,25 @@
         <f>IF(H32="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K32" s="50">
+        <f>IF(H32="","",RANK(H32,$H$15:$H$36,0)+COUNTIF($H$15:H32,H32)-1)</f>
+        <v/>
+      </c>
+      <c r="L32" s="51" t="n">
+        <v>18</v>
+      </c>
+      <c r="M32" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L32,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L32,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O32" s="48">
+        <f>IF(N32="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1" s="23">
       <c r="A33" s="43" t="n"/>
@@ -1661,6 +2037,25 @@
         <f>IF(H33="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K33" s="50">
+        <f>IF(H33="","",RANK(H33,$H$15:$H$36,0)+COUNTIF($H$15:H33,H33)-1)</f>
+        <v/>
+      </c>
+      <c r="L33" s="51" t="n">
+        <v>19</v>
+      </c>
+      <c r="M33" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L33,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L33,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O33" s="48">
+        <f>IF(N33="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1" s="23">
       <c r="A34" s="43" t="n"/>
@@ -1682,6 +2077,25 @@
         <f>IF(H34="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K34" s="50">
+        <f>IF(H34="","",RANK(H34,$H$15:$H$36,0)+COUNTIF($H$15:H34,H34)-1)</f>
+        <v/>
+      </c>
+      <c r="L34" s="51" t="n">
+        <v>20</v>
+      </c>
+      <c r="M34" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L34,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L34,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="48">
+        <f>IF(N34="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1" s="23">
       <c r="A35" s="43" t="n"/>
@@ -1703,10 +2117,48 @@
         <f>IF(H35="","",AVERAGE($H$15:$H$36))</f>
         <v/>
       </c>
+      <c r="K35" s="50">
+        <f>IF(H35="","",RANK(H35,$H$15:$H$36,0)+COUNTIF($H$15:H35,H35)-1)</f>
+        <v/>
+      </c>
+      <c r="L35" s="51" t="n">
+        <v>21</v>
+      </c>
+      <c r="M35" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L35,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L35,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O35" s="48">
+        <f>IF(N35="","",AVERAGE($N$15:$N$36))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="J36" s="48">
         <f>IF(H36="","",AVERAGE($H$15:$H$36))</f>
+        <v/>
+      </c>
+      <c r="K36" s="50">
+        <f>IF(H36="","",RANK(H36,$H$15:$H$36,0)+COUNTIF($H$15:H36,H36)-1)</f>
+        <v/>
+      </c>
+      <c r="L36" s="51" t="n">
+        <v>22</v>
+      </c>
+      <c r="M36" s="52">
+        <f>IFERROR(INDEX($A$15:$A$36,MATCH(L36,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="48">
+        <f>IFERROR(INDEX($H$15:$H$36,MATCH(L36,$K$15:$K$36,0)),"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="48">
+        <f>IF(N36="","",AVERAGE($N$15:$N$36))</f>
         <v/>
       </c>
     </row>

</xml_diff>